<commit_message>
Add data processing scripts and update Excel files for REDCap integration
</commit_message>
<xml_diff>
--- a/code_book/Variables Actualizada.xlsx
+++ b/code_book/Variables Actualizada.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreapaolasolispazmino/Library/CloudStorage/GoogleDrive-paosolpaz18@gmail.com/Mi unidad/Research/PHD/Projeto/1. Base de datos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luis_\Desktop\github\CATALINA_PROJECT\code_book\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA53911E-20E9-B740-A0A9-56163A0804FA}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11827A2E-D864-4ACB-951B-A8D30F573CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22040" yWindow="620" windowWidth="22040" windowHeight="14220" xr2:uid="{C9D495FD-1166-C646-BE06-9E489D4A3A9A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C9D495FD-1166-C646-BE06-9E489D4A3A9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="179021"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="122">
   <si>
     <t>record_id</t>
   </si>
@@ -385,13 +396,19 @@
   </si>
   <si>
     <t>1= N1a</t>
+  </si>
+  <si>
+    <t>0 no exicision</t>
+  </si>
+  <si>
+    <t>0 no RAI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -467,34 +484,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -513,9 +527,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -553,7 +567,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -659,7 +673,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -801,7 +815,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -810,177 +824,177 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358B9FBF-5B39-A04F-9E3D-D1C51686B25B}">
   <dimension ref="A1:AX20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="7"/>
+    <col min="1" max="1" width="10.83203125"/>
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="8" max="8" width="25.83203125" customWidth="1"/>
     <col min="10" max="10" width="22.6640625" customWidth="1"/>
     <col min="11" max="11" width="20" customWidth="1"/>
     <col min="12" max="12" width="17" customWidth="1"/>
-    <col min="16" max="16" width="10.83203125" style="7"/>
-    <col min="26" max="28" width="10.83203125" style="7"/>
+    <col min="16" max="16" width="10.83203125"/>
+    <col min="26" max="28" width="10.83203125"/>
     <col min="33" max="33" width="17" customWidth="1"/>
-    <col min="39" max="40" width="15.5" style="7" customWidth="1"/>
-    <col min="45" max="45" width="10.83203125" style="7"/>
+    <col min="39" max="40" width="15.5" customWidth="1"/>
+    <col min="45" max="45" width="10.83203125"/>
     <col min="49" max="49" width="24.83203125" customWidth="1"/>
     <col min="50" max="50" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" s="1" customFormat="1" ht="85" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:50" ht="62">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="V1" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Y1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AA1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AB1" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AD1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AE1" s="4" t="s">
+      <c r="AE1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AF1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AG1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AH1" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="AI1" s="5" t="s">
+      <c r="AI1" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="AJ1" s="4" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="AK1" s="5" t="s">
+      <c r="AK1" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="AL1" s="3" t="s">
+      <c r="AL1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AM1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="AN1" s="8" t="s">
+      <c r="AN1" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="AO1" s="9" t="s">
+      <c r="AO1" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="AP1" s="9" t="s">
+      <c r="AP1" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="AQ1" s="9" t="s">
+      <c r="AQ1" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="AR1" s="3" t="s">
+      <c r="AR1" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="AS1" s="9" t="s">
+      <c r="AS1" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="AT1" s="9" t="s">
+      <c r="AT1" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="AU1" s="6" t="s">
+      <c r="AU1" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="AV1" s="9" t="s">
+      <c r="AV1" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="AW1" s="3" t="s">
+      <c r="AW1" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="AX1" s="3" t="s">
+      <c r="AX1" s="2" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="1:50">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D2" t="s">
@@ -1004,16 +1018,16 @@
       <c r="K2" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="1" t="s">
         <v>29</v>
       </c>
       <c r="O2" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="10" t="s">
+      <c r="P2" s="1" t="s">
         <v>114</v>
       </c>
       <c r="Q2" t="s">
@@ -1031,19 +1045,19 @@
       <c r="Y2" t="s">
         <v>3</v>
       </c>
-      <c r="Z2" s="13" t="s">
+      <c r="Z2" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="AA2" s="13" t="s">
+      <c r="AA2" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="AB2" s="7" t="s">
+      <c r="AB2" t="s">
         <v>90</v>
       </c>
-      <c r="AC2" s="2" t="s">
+      <c r="AC2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AD2" s="1" t="s">
         <v>36</v>
       </c>
       <c r="AE2" t="s">
@@ -1067,15 +1081,15 @@
       <c r="AU2" t="s">
         <v>45</v>
       </c>
-      <c r="AW2" s="2" t="s">
+      <c r="AW2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AX2" s="2" t="s">
+      <c r="AX2" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:50">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D3" t="s">
@@ -1096,19 +1110,19 @@
       <c r="J3" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="1" t="s">
         <v>27</v>
       </c>
       <c r="O3" t="s">
         <v>4</v>
       </c>
-      <c r="P3" s="10" t="s">
+      <c r="P3" s="1" t="s">
         <v>115</v>
       </c>
       <c r="Q3" t="s">
@@ -1126,16 +1140,16 @@
       <c r="Y3" t="s">
         <v>4</v>
       </c>
-      <c r="Z3" s="13" t="s">
+      <c r="Z3" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="AA3" s="13" t="s">
+      <c r="AA3" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="AC3" s="2" t="s">
+      <c r="AC3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AD3" s="2" t="s">
+      <c r="AD3" s="1" t="s">
         <v>33</v>
       </c>
       <c r="AE3" t="s">
@@ -1159,14 +1173,14 @@
       <c r="AU3" t="s">
         <v>46</v>
       </c>
-      <c r="AW3" s="2" t="s">
+      <c r="AW3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="AX3" s="2" t="s">
+      <c r="AX3" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:50" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:50">
       <c r="F4" t="s">
         <v>63</v>
       </c>
@@ -1176,26 +1190,41 @@
       <c r="J4" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="P4" s="10"/>
-      <c r="Z4" s="13" t="s">
+      <c r="P4" s="1"/>
+      <c r="S4" t="s">
+        <v>120</v>
+      </c>
+      <c r="U4" t="s">
+        <v>120</v>
+      </c>
+      <c r="V4" t="s">
+        <v>120</v>
+      </c>
+      <c r="W4" t="s">
+        <v>120</v>
+      </c>
+      <c r="X4" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z4" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="AA4" s="7" t="s">
+      <c r="AA4" t="s">
         <v>118</v>
       </c>
-      <c r="AD4" s="2" t="s">
+      <c r="AD4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AE4" s="7" t="s">
+      <c r="AE4" t="s">
         <v>93</v>
       </c>
       <c r="AF4" t="s">
@@ -1204,119 +1233,122 @@
       <c r="AG4" t="s">
         <v>41</v>
       </c>
-      <c r="AW4" s="2" t="s">
+      <c r="AP4" t="s">
+        <v>121</v>
+      </c>
+      <c r="AW4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AX4" s="2" t="s">
+      <c r="AX4" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K5" s="2" t="s">
+    <row r="5" spans="1:50">
+      <c r="K5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Z5" s="13" t="s">
+      <c r="Z5" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="AA5" s="13" t="s">
+      <c r="AA5" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="AD5" s="2" t="s">
+      <c r="AD5" s="1" t="s">
         <v>35</v>
       </c>
       <c r="AG5" t="s">
         <v>42</v>
       </c>
-      <c r="AW5" s="2" t="s">
+      <c r="AW5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="AX5" s="2" t="s">
+      <c r="AX5" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K6" s="2" t="s">
+    <row r="6" spans="1:50">
+      <c r="K6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="Z6" s="13" t="s">
+      <c r="Z6" s="10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K7" s="2" t="s">
+    <row r="7" spans="1:50">
+      <c r="K7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="10"/>
-      <c r="AA7" s="14"/>
+      <c r="P7" s="1"/>
+      <c r="AA7" s="11"/>
       <c r="AJ7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K8" s="2" t="s">
+    <row r="8" spans="1:50">
+      <c r="K8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="P8" s="12"/>
-      <c r="AW8" s="2" t="s">
+      <c r="P8" s="9"/>
+      <c r="AW8" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K9" s="2" t="s">
+    <row r="9" spans="1:50">
+      <c r="K9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="P9" s="12"/>
+      <c r="P9" s="9"/>
       <c r="S9" t="s">
         <v>54</v>
       </c>
-      <c r="Z9" s="14"/>
-    </row>
-    <row r="10" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K10" s="2" t="s">
+      <c r="Z9" s="11"/>
+    </row>
+    <row r="10" spans="1:50">
+      <c r="K10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="P10" s="12"/>
-      <c r="Z10" s="14"/>
-    </row>
-    <row r="11" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K11" s="10" t="s">
+      <c r="P10" s="9"/>
+      <c r="Z10" s="11"/>
+    </row>
+    <row r="11" spans="1:50">
+      <c r="K11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="P11" s="12"/>
-      <c r="Z11" s="14"/>
-    </row>
-    <row r="12" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K12" s="10" t="s">
+      <c r="P11" s="9"/>
+      <c r="Z11" s="11"/>
+    </row>
+    <row r="12" spans="1:50">
+      <c r="K12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="Z12" s="14"/>
-    </row>
-    <row r="13" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K13" s="11" t="s">
+      <c r="Z12" s="11"/>
+    </row>
+    <row r="13" spans="1:50">
+      <c r="K13" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="Z13" s="14"/>
-    </row>
-    <row r="14" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K14" s="11" t="s">
+      <c r="Z13" s="11"/>
+    </row>
+    <row r="14" spans="1:50">
+      <c r="K14" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="Z14" s="14"/>
-    </row>
-    <row r="15" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="K15" s="2"/>
-      <c r="Z15" s="14"/>
-    </row>
-    <row r="16" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="AB16" s="13"/>
-    </row>
-    <row r="17" spans="28:32" x14ac:dyDescent="0.2">
-      <c r="AB17" s="13"/>
-    </row>
-    <row r="18" spans="28:32" x14ac:dyDescent="0.2">
-      <c r="AB18" s="13"/>
-    </row>
-    <row r="20" spans="28:32" x14ac:dyDescent="0.2">
+      <c r="Z14" s="11"/>
+    </row>
+    <row r="15" spans="1:50">
+      <c r="K15" s="1"/>
+      <c r="Z15" s="11"/>
+    </row>
+    <row r="16" spans="1:50">
+      <c r="AB16" s="10"/>
+    </row>
+    <row r="17" spans="28:32">
+      <c r="AB17" s="10"/>
+    </row>
+    <row r="18" spans="28:32">
+      <c r="AB18" s="10"/>
+    </row>
+    <row r="20" spans="28:32">
       <c r="AF20" t="s">
         <v>54</v>
       </c>

</xml_diff>